<commit_message>
feat: Enhance river outfall status visualizer with new elevation fields and input template
- Added 'bed_elev' and 'levee_elev' fields to FIELD_ALIASES for better data representation.
- Updated the read and write functions to handle new elevation fields in Excel files.
- Introduced a new script to generate an input template Excel file with detailed instructions for users.
- Created a comprehensive guide for filling out the input template, including examples and requirements.
- Added a new Excel template file for user input, ensuring clarity and ease of use.
</commit_message>
<xml_diff>
--- a/river-outfall-status-visualizer/assets/examples/example-river-sample.xlsx
+++ b/river-outfall-status-visualizer/assets/examples/example-river-sample.xlsx
@@ -8,7 +8,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="163">
   <si>
     <t xml:space="preserve">排河口编号</t>
   </si>
@@ -23,6 +23,12 @@
   </si>
   <si>
     <t xml:space="preserve">底高程</t>
+  </si>
+  <si>
+    <t xml:space="preserve">河底高程</t>
+  </si>
+  <si>
+    <t xml:space="preserve">堤顶高程</t>
   </si>
   <si>
     <t xml:space="preserve">里程</t>
@@ -578,1724 +584,2030 @@
       <c r="M1" t="s">
         <v>12</v>
       </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="2">
       <c r="F2">
+        <v>18.2</v>
+      </c>
+      <c r="G2">
+        <v>25.4</v>
+      </c>
+      <c r="H2">
         <v>0</v>
       </c>
-      <c r="I2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J2">
+      <c r="K2" t="s">
+        <v>15</v>
+      </c>
+      <c r="L2">
         <v>22.1</v>
       </c>
-      <c r="K2">
+      <c r="M2">
         <v>21.7</v>
       </c>
-      <c r="L2">
+      <c r="N2">
         <v>23.05</v>
       </c>
-      <c r="M2">
+      <c r="O2">
         <v>23.85</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E3">
         <v>22.65</v>
       </c>
       <c r="F3">
+        <v>18.2</v>
+      </c>
+      <c r="G3">
+        <v>25.4</v>
+      </c>
+      <c r="H3">
         <v>180</v>
       </c>
-      <c r="G3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H3" t="s">
-        <v>19</v>
-      </c>
-      <c r="J3">
+      <c r="I3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" t="s">
+        <v>21</v>
+      </c>
+      <c r="L3">
         <v>22.1</v>
       </c>
-      <c r="K3">
+      <c r="M3">
         <v>21.7</v>
       </c>
-      <c r="L3">
+      <c r="N3">
         <v>23.05</v>
       </c>
-      <c r="M3">
+      <c r="O3">
         <v>23.85</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E4">
         <v>21.45</v>
       </c>
       <c r="F4">
+        <v>18.2</v>
+      </c>
+      <c r="G4">
+        <v>25.4</v>
+      </c>
+      <c r="H4">
         <v>430</v>
       </c>
-      <c r="G4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H4" t="s">
-        <v>19</v>
-      </c>
-      <c r="J4">
+      <c r="I4" t="s">
+        <v>26</v>
+      </c>
+      <c r="J4" t="s">
+        <v>21</v>
+      </c>
+      <c r="L4">
         <v>22.1</v>
       </c>
-      <c r="K4">
+      <c r="M4">
         <v>21.7</v>
       </c>
-      <c r="L4">
+      <c r="N4">
         <v>23.05</v>
       </c>
-      <c r="M4">
+      <c r="O4">
         <v>23.85</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E5">
         <v>22.05</v>
       </c>
       <c r="F5">
+        <v>18.2</v>
+      </c>
+      <c r="G5">
+        <v>25.4</v>
+      </c>
+      <c r="H5">
         <v>710</v>
       </c>
-      <c r="G5" t="s">
-        <v>18</v>
-      </c>
-      <c r="H5" t="s">
-        <v>19</v>
-      </c>
-      <c r="J5">
+      <c r="I5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J5" t="s">
+        <v>21</v>
+      </c>
+      <c r="L5">
         <v>22.1</v>
       </c>
-      <c r="K5">
+      <c r="M5">
         <v>21.7</v>
       </c>
-      <c r="L5">
+      <c r="N5">
         <v>23.05</v>
       </c>
-      <c r="M5">
+      <c r="O5">
         <v>23.85</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E6">
         <v>23.05</v>
       </c>
       <c r="F6">
+        <v>18.2</v>
+      </c>
+      <c r="G6">
+        <v>25.4</v>
+      </c>
+      <c r="H6">
         <v>980</v>
       </c>
-      <c r="G6" t="s">
-        <v>24</v>
-      </c>
-      <c r="H6" t="s">
-        <v>19</v>
-      </c>
-      <c r="J6">
+      <c r="I6" t="s">
+        <v>26</v>
+      </c>
+      <c r="J6" t="s">
+        <v>21</v>
+      </c>
+      <c r="L6">
         <v>22.1</v>
       </c>
-      <c r="K6">
+      <c r="M6">
         <v>21.7</v>
       </c>
-      <c r="L6">
+      <c r="N6">
         <v>23.05</v>
       </c>
-      <c r="M6">
+      <c r="O6">
         <v>23.85</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B7" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C7" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D7" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E7">
         <v>21</v>
       </c>
       <c r="F7">
+        <v>18.2</v>
+      </c>
+      <c r="G7">
+        <v>25.4</v>
+      </c>
+      <c r="H7">
         <v>1260</v>
       </c>
-      <c r="G7" t="s">
-        <v>24</v>
-      </c>
-      <c r="H7" t="s">
-        <v>19</v>
-      </c>
-      <c r="J7">
+      <c r="I7" t="s">
+        <v>26</v>
+      </c>
+      <c r="J7" t="s">
+        <v>21</v>
+      </c>
+      <c r="L7">
         <v>22.1</v>
       </c>
-      <c r="K7">
+      <c r="M7">
         <v>21.7</v>
       </c>
-      <c r="L7">
+      <c r="N7">
         <v>23.05</v>
       </c>
-      <c r="M7">
+      <c r="O7">
         <v>23.85</v>
       </c>
     </row>
     <row r="8">
       <c r="F8">
+        <v>17.35</v>
+      </c>
+      <c r="G8">
+        <v>24.75</v>
+      </c>
+      <c r="H8">
         <v>1500</v>
       </c>
-      <c r="I8" t="s">
-        <v>37</v>
-      </c>
-      <c r="J8">
+      <c r="K8" t="s">
+        <v>39</v>
+      </c>
+      <c r="L8">
         <v>21.15</v>
       </c>
-      <c r="K8">
+      <c r="M8">
         <v>20.75</v>
       </c>
-      <c r="L8">
+      <c r="N8">
         <v>22.5</v>
       </c>
-      <c r="M8">
+      <c r="O8">
         <v>23.2</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E9">
         <v>20.9</v>
       </c>
       <c r="F9">
+        <v>17.35</v>
+      </c>
+      <c r="G9">
+        <v>24.75</v>
+      </c>
+      <c r="H9">
         <v>1580</v>
       </c>
-      <c r="G9" t="s">
-        <v>24</v>
-      </c>
-      <c r="H9" t="s">
-        <v>19</v>
-      </c>
-      <c r="J9">
+      <c r="I9" t="s">
+        <v>26</v>
+      </c>
+      <c r="J9" t="s">
+        <v>21</v>
+      </c>
+      <c r="L9">
         <v>21.15</v>
       </c>
-      <c r="K9">
+      <c r="M9">
         <v>20.75</v>
       </c>
-      <c r="L9">
+      <c r="N9">
         <v>22.5</v>
       </c>
-      <c r="M9">
+      <c r="O9">
         <v>23.2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E10">
         <v>21.6</v>
       </c>
       <c r="F10">
+        <v>17.35</v>
+      </c>
+      <c r="G10">
+        <v>24.75</v>
+      </c>
+      <c r="H10">
         <v>1870</v>
       </c>
-      <c r="G10" t="s">
-        <v>18</v>
-      </c>
-      <c r="H10" t="s">
-        <v>19</v>
-      </c>
-      <c r="J10">
+      <c r="I10" t="s">
+        <v>20</v>
+      </c>
+      <c r="J10" t="s">
+        <v>21</v>
+      </c>
+      <c r="L10">
         <v>21.15</v>
       </c>
-      <c r="K10">
+      <c r="M10">
         <v>20.75</v>
       </c>
-      <c r="L10">
+      <c r="N10">
         <v>22.5</v>
       </c>
-      <c r="M10">
+      <c r="O10">
         <v>23.2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B11" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C11" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D11" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E11">
         <v>19.7</v>
       </c>
       <c r="F11">
+        <v>17.35</v>
+      </c>
+      <c r="G11">
+        <v>24.75</v>
+      </c>
+      <c r="H11">
         <v>2140</v>
       </c>
-      <c r="G11" t="s">
-        <v>24</v>
-      </c>
-      <c r="H11" t="s">
-        <v>19</v>
-      </c>
-      <c r="J11">
+      <c r="I11" t="s">
+        <v>26</v>
+      </c>
+      <c r="J11" t="s">
+        <v>21</v>
+      </c>
+      <c r="L11">
         <v>21.15</v>
       </c>
-      <c r="K11">
+      <c r="M11">
         <v>20.75</v>
       </c>
-      <c r="L11">
+      <c r="N11">
         <v>22.5</v>
       </c>
-      <c r="M11">
+      <c r="O11">
         <v>23.2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B12" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C12" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D12" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E12">
         <v>22.3</v>
       </c>
       <c r="F12">
+        <v>17.35</v>
+      </c>
+      <c r="G12">
+        <v>24.75</v>
+      </c>
+      <c r="H12">
         <v>2430</v>
       </c>
-      <c r="G12" t="s">
-        <v>18</v>
-      </c>
-      <c r="H12" t="s">
-        <v>19</v>
-      </c>
-      <c r="J12">
+      <c r="I12" t="s">
+        <v>20</v>
+      </c>
+      <c r="J12" t="s">
+        <v>21</v>
+      </c>
+      <c r="L12">
         <v>21.15</v>
       </c>
-      <c r="K12">
+      <c r="M12">
         <v>20.75</v>
       </c>
-      <c r="L12">
+      <c r="N12">
         <v>22.5</v>
       </c>
-      <c r="M12">
+      <c r="O12">
         <v>23.2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B13" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C13" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D13" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E13">
         <v>21.3</v>
       </c>
       <c r="F13">
+        <v>17.35</v>
+      </c>
+      <c r="G13">
+        <v>24.75</v>
+      </c>
+      <c r="H13">
         <v>2720</v>
       </c>
-      <c r="G13" t="s">
-        <v>18</v>
-      </c>
-      <c r="H13" t="s">
-        <v>19</v>
-      </c>
-      <c r="J13">
+      <c r="I13" t="s">
+        <v>20</v>
+      </c>
+      <c r="J13" t="s">
+        <v>21</v>
+      </c>
+      <c r="L13">
         <v>21.15</v>
       </c>
-      <c r="K13">
+      <c r="M13">
         <v>20.75</v>
       </c>
-      <c r="L13">
+      <c r="N13">
         <v>22.5</v>
       </c>
-      <c r="M13">
+      <c r="O13">
         <v>23.2</v>
       </c>
     </row>
     <row r="14">
       <c r="F14">
+        <v>16.4</v>
+      </c>
+      <c r="G14">
+        <v>23.9</v>
+      </c>
+      <c r="H14">
         <v>2900</v>
       </c>
-      <c r="I14" t="s">
-        <v>58</v>
-      </c>
-      <c r="J14">
+      <c r="K14" t="s">
+        <v>60</v>
+      </c>
+      <c r="L14">
         <v>20.2</v>
       </c>
-      <c r="K14">
+      <c r="M14">
         <v>19.75</v>
       </c>
-      <c r="L14">
+      <c r="N14">
         <v>21.55</v>
       </c>
-      <c r="M14">
+      <c r="O14">
         <v>22.35</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B15" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C15" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D15" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E15">
         <v>19.35</v>
       </c>
       <c r="F15">
+        <v>16.4</v>
+      </c>
+      <c r="G15">
+        <v>23.9</v>
+      </c>
+      <c r="H15">
         <v>3050</v>
       </c>
-      <c r="G15" t="s">
-        <v>18</v>
-      </c>
-      <c r="H15" t="s">
-        <v>19</v>
-      </c>
-      <c r="J15">
+      <c r="I15" t="s">
+        <v>20</v>
+      </c>
+      <c r="J15" t="s">
+        <v>21</v>
+      </c>
+      <c r="L15">
         <v>20.2</v>
       </c>
-      <c r="K15">
+      <c r="M15">
         <v>19.75</v>
       </c>
-      <c r="L15">
+      <c r="N15">
         <v>21.55</v>
       </c>
-      <c r="M15">
+      <c r="O15">
         <v>22.35</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B16" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C16" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D16" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E16">
         <v>19.8</v>
       </c>
       <c r="F16">
+        <v>16.4</v>
+      </c>
+      <c r="G16">
+        <v>23.9</v>
+      </c>
+      <c r="H16">
         <v>3340</v>
       </c>
-      <c r="G16" t="s">
-        <v>24</v>
-      </c>
-      <c r="H16" t="s">
-        <v>19</v>
-      </c>
-      <c r="J16">
+      <c r="I16" t="s">
+        <v>26</v>
+      </c>
+      <c r="J16" t="s">
+        <v>21</v>
+      </c>
+      <c r="L16">
         <v>20.2</v>
       </c>
-      <c r="K16">
+      <c r="M16">
         <v>19.75</v>
       </c>
-      <c r="L16">
+      <c r="N16">
         <v>21.55</v>
       </c>
-      <c r="M16">
+      <c r="O16">
         <v>22.35</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C17" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D17" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E17">
         <v>20.9</v>
       </c>
       <c r="F17">
+        <v>16.4</v>
+      </c>
+      <c r="G17">
+        <v>23.9</v>
+      </c>
+      <c r="H17">
         <v>3620</v>
       </c>
-      <c r="G17" t="s">
-        <v>18</v>
-      </c>
-      <c r="H17" t="s">
-        <v>19</v>
-      </c>
-      <c r="J17">
+      <c r="I17" t="s">
+        <v>20</v>
+      </c>
+      <c r="J17" t="s">
+        <v>21</v>
+      </c>
+      <c r="L17">
         <v>20.2</v>
       </c>
-      <c r="K17">
+      <c r="M17">
         <v>19.75</v>
       </c>
-      <c r="L17">
+      <c r="N17">
         <v>21.55</v>
       </c>
-      <c r="M17">
+      <c r="O17">
         <v>22.35</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C18" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D18" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E18">
         <v>18.9</v>
       </c>
       <c r="F18">
+        <v>16.4</v>
+      </c>
+      <c r="G18">
+        <v>23.9</v>
+      </c>
+      <c r="H18">
         <v>3890</v>
       </c>
-      <c r="G18" t="s">
-        <v>24</v>
-      </c>
-      <c r="H18" t="s">
-        <v>19</v>
-      </c>
-      <c r="J18">
+      <c r="I18" t="s">
+        <v>26</v>
+      </c>
+      <c r="J18" t="s">
+        <v>21</v>
+      </c>
+      <c r="L18">
         <v>20.2</v>
       </c>
-      <c r="K18">
+      <c r="M18">
         <v>19.75</v>
       </c>
-      <c r="L18">
+      <c r="N18">
         <v>21.55</v>
       </c>
-      <c r="M18">
+      <c r="O18">
         <v>22.35</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B19" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C19" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D19" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E19">
         <v>20.2</v>
       </c>
       <c r="F19">
+        <v>16.4</v>
+      </c>
+      <c r="G19">
+        <v>23.9</v>
+      </c>
+      <c r="H19">
         <v>4170</v>
       </c>
-      <c r="G19" t="s">
-        <v>24</v>
-      </c>
-      <c r="H19" t="s">
-        <v>19</v>
-      </c>
-      <c r="J19">
+      <c r="I19" t="s">
+        <v>26</v>
+      </c>
+      <c r="J19" t="s">
+        <v>21</v>
+      </c>
+      <c r="L19">
         <v>20.2</v>
       </c>
-      <c r="K19">
+      <c r="M19">
         <v>19.75</v>
       </c>
-      <c r="L19">
+      <c r="N19">
         <v>21.55</v>
       </c>
-      <c r="M19">
+      <c r="O19">
         <v>22.35</v>
       </c>
     </row>
     <row r="20">
       <c r="F20">
+        <v>15.5</v>
+      </c>
+      <c r="G20">
+        <v>23.05</v>
+      </c>
+      <c r="H20">
         <v>4200</v>
       </c>
-      <c r="I20" t="s">
-        <v>77</v>
-      </c>
-      <c r="J20">
+      <c r="K20" t="s">
+        <v>79</v>
+      </c>
+      <c r="L20">
         <v>19.2</v>
       </c>
-      <c r="K20">
+      <c r="M20">
         <v>18.7</v>
       </c>
-      <c r="L20">
+      <c r="N20">
         <v>20.8</v>
       </c>
-      <c r="M20">
+      <c r="O20">
         <v>21.7</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B21" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C21" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D21" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E21">
         <v>20.45</v>
       </c>
       <c r="F21">
+        <v>15.5</v>
+      </c>
+      <c r="G21">
+        <v>23.05</v>
+      </c>
+      <c r="H21">
         <v>4470</v>
       </c>
-      <c r="G21" t="s">
-        <v>24</v>
-      </c>
-      <c r="H21" t="s">
-        <v>19</v>
-      </c>
-      <c r="J21">
+      <c r="I21" t="s">
+        <v>26</v>
+      </c>
+      <c r="J21" t="s">
+        <v>21</v>
+      </c>
+      <c r="L21">
         <v>19.2</v>
       </c>
-      <c r="K21">
+      <c r="M21">
         <v>18.7</v>
       </c>
-      <c r="L21">
+      <c r="N21">
         <v>20.8</v>
       </c>
-      <c r="M21">
+      <c r="O21">
         <v>21.7</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B22" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C22" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D22" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E22">
         <v>17.5</v>
       </c>
       <c r="F22">
+        <v>15.5</v>
+      </c>
+      <c r="G22">
+        <v>23.05</v>
+      </c>
+      <c r="H22">
         <v>4760</v>
       </c>
-      <c r="G22" t="s">
-        <v>18</v>
-      </c>
-      <c r="H22" t="s">
-        <v>19</v>
-      </c>
-      <c r="J22">
+      <c r="I22" t="s">
+        <v>20</v>
+      </c>
+      <c r="J22" t="s">
+        <v>21</v>
+      </c>
+      <c r="L22">
         <v>19.2</v>
       </c>
-      <c r="K22">
+      <c r="M22">
         <v>18.7</v>
       </c>
-      <c r="L22">
+      <c r="N22">
         <v>20.8</v>
       </c>
-      <c r="M22">
+      <c r="O22">
         <v>21.7</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B23" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C23" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D23" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E23">
         <v>18.95</v>
       </c>
       <c r="F23">
+        <v>15.5</v>
+      </c>
+      <c r="G23">
+        <v>23.05</v>
+      </c>
+      <c r="H23">
         <v>5060</v>
       </c>
-      <c r="G23" t="s">
-        <v>24</v>
-      </c>
-      <c r="H23" t="s">
-        <v>19</v>
-      </c>
-      <c r="J23">
+      <c r="I23" t="s">
+        <v>26</v>
+      </c>
+      <c r="J23" t="s">
+        <v>21</v>
+      </c>
+      <c r="L23">
         <v>19.2</v>
       </c>
-      <c r="K23">
+      <c r="M23">
         <v>18.7</v>
       </c>
-      <c r="L23">
+      <c r="N23">
         <v>20.8</v>
       </c>
-      <c r="M23">
+      <c r="O23">
         <v>21.7</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B24" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C24" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D24" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E24">
         <v>19.45</v>
       </c>
       <c r="F24">
+        <v>15.5</v>
+      </c>
+      <c r="G24">
+        <v>23.05</v>
+      </c>
+      <c r="H24">
         <v>5360</v>
       </c>
-      <c r="G24" t="s">
-        <v>18</v>
-      </c>
-      <c r="H24" t="s">
-        <v>19</v>
-      </c>
-      <c r="J24">
+      <c r="I24" t="s">
+        <v>20</v>
+      </c>
+      <c r="J24" t="s">
+        <v>21</v>
+      </c>
+      <c r="L24">
         <v>19.2</v>
       </c>
-      <c r="K24">
+      <c r="M24">
         <v>18.7</v>
       </c>
-      <c r="L24">
+      <c r="N24">
         <v>20.8</v>
       </c>
-      <c r="M24">
+      <c r="O24">
         <v>21.7</v>
       </c>
     </row>
     <row r="25">
       <c r="F25">
+        <v>14.65</v>
+      </c>
+      <c r="G25">
+        <v>22.1</v>
+      </c>
+      <c r="H25">
         <v>5600</v>
       </c>
-      <c r="I25" t="s">
-        <v>92</v>
-      </c>
-      <c r="J25">
+      <c r="K25" t="s">
+        <v>94</v>
+      </c>
+      <c r="L25">
         <v>18.25</v>
       </c>
-      <c r="K25">
+      <c r="M25">
         <v>17.8</v>
       </c>
-      <c r="L25">
+      <c r="N25">
         <v>19.95</v>
       </c>
-      <c r="M25">
+      <c r="O25">
         <v>20.9</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B26" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C26" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D26" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E26">
         <v>17.25</v>
       </c>
       <c r="F26">
+        <v>14.65</v>
+      </c>
+      <c r="G26">
+        <v>22.1</v>
+      </c>
+      <c r="H26">
         <v>5660</v>
       </c>
-      <c r="G26" t="s">
-        <v>18</v>
-      </c>
-      <c r="H26" t="s">
-        <v>19</v>
-      </c>
-      <c r="J26">
+      <c r="I26" t="s">
+        <v>20</v>
+      </c>
+      <c r="J26" t="s">
+        <v>21</v>
+      </c>
+      <c r="L26">
         <v>18.25</v>
       </c>
-      <c r="K26">
+      <c r="M26">
         <v>17.8</v>
       </c>
-      <c r="L26">
+      <c r="N26">
         <v>19.95</v>
       </c>
-      <c r="M26">
+      <c r="O26">
         <v>20.9</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B27" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C27" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D27" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E27">
         <v>18.75</v>
       </c>
       <c r="F27">
+        <v>14.65</v>
+      </c>
+      <c r="G27">
+        <v>22.1</v>
+      </c>
+      <c r="H27">
         <v>5960</v>
       </c>
-      <c r="G27" t="s">
-        <v>18</v>
-      </c>
-      <c r="H27" t="s">
-        <v>19</v>
-      </c>
-      <c r="J27">
+      <c r="I27" t="s">
+        <v>20</v>
+      </c>
+      <c r="J27" t="s">
+        <v>21</v>
+      </c>
+      <c r="L27">
         <v>18.25</v>
       </c>
-      <c r="K27">
+      <c r="M27">
         <v>17.8</v>
       </c>
-      <c r="L27">
+      <c r="N27">
         <v>19.95</v>
       </c>
-      <c r="M27">
+      <c r="O27">
         <v>20.9</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B28" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C28" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D28" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E28">
         <v>17.55</v>
       </c>
       <c r="F28">
+        <v>14.65</v>
+      </c>
+      <c r="G28">
+        <v>22.1</v>
+      </c>
+      <c r="H28">
         <v>6260</v>
       </c>
-      <c r="G28" t="s">
-        <v>24</v>
-      </c>
-      <c r="H28" t="s">
-        <v>19</v>
-      </c>
-      <c r="J28">
+      <c r="I28" t="s">
+        <v>26</v>
+      </c>
+      <c r="J28" t="s">
+        <v>21</v>
+      </c>
+      <c r="L28">
         <v>18.25</v>
       </c>
-      <c r="K28">
+      <c r="M28">
         <v>17.8</v>
       </c>
-      <c r="L28">
+      <c r="N28">
         <v>19.95</v>
       </c>
-      <c r="M28">
+      <c r="O28">
         <v>20.9</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B29" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C29" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E29">
         <v>18.15</v>
       </c>
       <c r="F29">
+        <v>14.65</v>
+      </c>
+      <c r="G29">
+        <v>22.1</v>
+      </c>
+      <c r="H29">
         <v>6560</v>
       </c>
-      <c r="G29" t="s">
-        <v>18</v>
-      </c>
-      <c r="H29" t="s">
-        <v>19</v>
-      </c>
-      <c r="J29">
+      <c r="I29" t="s">
+        <v>20</v>
+      </c>
+      <c r="J29" t="s">
+        <v>21</v>
+      </c>
+      <c r="L29">
         <v>18.25</v>
       </c>
-      <c r="K29">
+      <c r="M29">
         <v>17.8</v>
       </c>
-      <c r="L29">
+      <c r="N29">
         <v>19.95</v>
       </c>
-      <c r="M29">
+      <c r="O29">
         <v>20.9</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B30" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C30" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D30" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E30">
         <v>19.15</v>
       </c>
       <c r="F30">
+        <v>14.65</v>
+      </c>
+      <c r="G30">
+        <v>22.1</v>
+      </c>
+      <c r="H30">
         <v>6860</v>
       </c>
-      <c r="G30" t="s">
-        <v>24</v>
-      </c>
-      <c r="H30" t="s">
-        <v>19</v>
-      </c>
-      <c r="J30">
+      <c r="I30" t="s">
+        <v>26</v>
+      </c>
+      <c r="J30" t="s">
+        <v>21</v>
+      </c>
+      <c r="L30">
         <v>18.25</v>
       </c>
-      <c r="K30">
+      <c r="M30">
         <v>17.8</v>
       </c>
-      <c r="L30">
+      <c r="N30">
         <v>19.95</v>
       </c>
-      <c r="M30">
+      <c r="O30">
         <v>20.9</v>
       </c>
     </row>
     <row r="31">
       <c r="F31">
+        <v>13.9</v>
+      </c>
+      <c r="G31">
+        <v>21.15</v>
+      </c>
+      <c r="H31">
         <v>7100</v>
       </c>
-      <c r="I31" t="s">
-        <v>108</v>
-      </c>
-      <c r="J31">
+      <c r="K31" t="s">
+        <v>110</v>
+      </c>
+      <c r="L31">
         <v>17.4</v>
       </c>
-      <c r="K31">
+      <c r="M31">
         <v>16.95</v>
       </c>
-      <c r="L31">
+      <c r="N31">
         <v>18.95</v>
       </c>
-      <c r="M31">
+      <c r="O31">
         <v>20.05</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B32" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C32" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D32" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E32">
         <v>16.25</v>
       </c>
       <c r="F32">
+        <v>13.9</v>
+      </c>
+      <c r="G32">
+        <v>21.15</v>
+      </c>
+      <c r="H32">
         <v>7160</v>
       </c>
-      <c r="G32" t="s">
-        <v>24</v>
-      </c>
-      <c r="H32" t="s">
-        <v>19</v>
-      </c>
-      <c r="J32">
+      <c r="I32" t="s">
+        <v>26</v>
+      </c>
+      <c r="J32" t="s">
+        <v>21</v>
+      </c>
+      <c r="L32">
         <v>17.4</v>
       </c>
-      <c r="K32">
+      <c r="M32">
         <v>16.95</v>
       </c>
-      <c r="L32">
+      <c r="N32">
         <v>18.95</v>
       </c>
-      <c r="M32">
+      <c r="O32">
         <v>20.05</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B33" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C33" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D33" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E33">
         <v>17.1</v>
       </c>
       <c r="F33">
+        <v>13.9</v>
+      </c>
+      <c r="G33">
+        <v>21.15</v>
+      </c>
+      <c r="H33">
         <v>7460</v>
       </c>
-      <c r="G33" t="s">
-        <v>24</v>
-      </c>
-      <c r="H33" t="s">
-        <v>19</v>
-      </c>
-      <c r="J33">
+      <c r="I33" t="s">
+        <v>26</v>
+      </c>
+      <c r="J33" t="s">
+        <v>21</v>
+      </c>
+      <c r="L33">
         <v>17.4</v>
       </c>
-      <c r="K33">
+      <c r="M33">
         <v>16.95</v>
       </c>
-      <c r="L33">
+      <c r="N33">
         <v>18.95</v>
       </c>
-      <c r="M33">
+      <c r="O33">
         <v>20.05</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B34" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C34" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D34" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E34">
         <v>17.8</v>
       </c>
       <c r="F34">
+        <v>13.9</v>
+      </c>
+      <c r="G34">
+        <v>21.15</v>
+      </c>
+      <c r="H34">
         <v>7760</v>
       </c>
-      <c r="G34" t="s">
-        <v>18</v>
-      </c>
-      <c r="H34" t="s">
-        <v>19</v>
-      </c>
-      <c r="J34">
+      <c r="I34" t="s">
+        <v>20</v>
+      </c>
+      <c r="J34" t="s">
+        <v>21</v>
+      </c>
+      <c r="L34">
         <v>17.4</v>
       </c>
-      <c r="K34">
+      <c r="M34">
         <v>16.95</v>
       </c>
-      <c r="L34">
+      <c r="N34">
         <v>18.95</v>
       </c>
-      <c r="M34">
+      <c r="O34">
         <v>20.05</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B35" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C35" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D35" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E35">
         <v>15.9</v>
       </c>
       <c r="F35">
+        <v>13.9</v>
+      </c>
+      <c r="G35">
+        <v>21.15</v>
+      </c>
+      <c r="H35">
         <v>8060</v>
       </c>
-      <c r="G35" t="s">
-        <v>24</v>
-      </c>
-      <c r="H35" t="s">
-        <v>19</v>
-      </c>
-      <c r="J35">
+      <c r="I35" t="s">
+        <v>26</v>
+      </c>
+      <c r="J35" t="s">
+        <v>21</v>
+      </c>
+      <c r="L35">
         <v>17.4</v>
       </c>
-      <c r="K35">
+      <c r="M35">
         <v>16.95</v>
       </c>
-      <c r="L35">
+      <c r="N35">
         <v>18.95</v>
       </c>
-      <c r="M35">
+      <c r="O35">
         <v>20.05</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B36" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C36" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D36" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E36">
         <v>18.5</v>
       </c>
       <c r="F36">
+        <v>13.9</v>
+      </c>
+      <c r="G36">
+        <v>21.15</v>
+      </c>
+      <c r="H36">
         <v>8360</v>
       </c>
-      <c r="G36" t="s">
-        <v>18</v>
-      </c>
-      <c r="H36" t="s">
-        <v>19</v>
-      </c>
-      <c r="J36">
+      <c r="I36" t="s">
+        <v>20</v>
+      </c>
+      <c r="J36" t="s">
+        <v>21</v>
+      </c>
+      <c r="L36">
         <v>17.4</v>
       </c>
-      <c r="K36">
+      <c r="M36">
         <v>16.95</v>
       </c>
-      <c r="L36">
+      <c r="N36">
         <v>18.95</v>
       </c>
-      <c r="M36">
+      <c r="O36">
         <v>20.05</v>
       </c>
     </row>
     <row r="37">
       <c r="F37">
+        <v>13.1</v>
+      </c>
+      <c r="G37">
+        <v>20.15</v>
+      </c>
+      <c r="H37">
         <v>8600</v>
       </c>
-      <c r="I37" t="s">
-        <v>124</v>
-      </c>
-      <c r="J37">
+      <c r="K37" t="s">
+        <v>126</v>
+      </c>
+      <c r="L37">
         <v>16.55</v>
       </c>
-      <c r="K37">
+      <c r="M37">
         <v>16.05</v>
       </c>
-      <c r="L37">
+      <c r="N37">
         <v>17.9</v>
       </c>
-      <c r="M37">
+      <c r="O37">
         <v>18.95</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B38" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C38" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D38" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E38">
         <v>16.6</v>
       </c>
       <c r="F38">
+        <v>13.1</v>
+      </c>
+      <c r="G38">
+        <v>20.15</v>
+      </c>
+      <c r="H38">
         <v>8660</v>
       </c>
-      <c r="G38" t="s">
-        <v>18</v>
-      </c>
-      <c r="H38" t="s">
-        <v>19</v>
-      </c>
-      <c r="J38">
+      <c r="I38" t="s">
+        <v>20</v>
+      </c>
+      <c r="J38" t="s">
+        <v>21</v>
+      </c>
+      <c r="L38">
         <v>16.55</v>
       </c>
-      <c r="K38">
+      <c r="M38">
         <v>16.05</v>
       </c>
-      <c r="L38">
+      <c r="N38">
         <v>17.9</v>
       </c>
-      <c r="M38">
+      <c r="O38">
         <v>18.95</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B39" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C39" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D39" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E39">
         <v>15.65</v>
       </c>
       <c r="F39">
+        <v>13.1</v>
+      </c>
+      <c r="G39">
+        <v>20.15</v>
+      </c>
+      <c r="H39">
         <v>8980</v>
       </c>
-      <c r="G39" t="s">
-        <v>18</v>
-      </c>
-      <c r="H39" t="s">
-        <v>19</v>
-      </c>
-      <c r="J39">
+      <c r="I39" t="s">
+        <v>20</v>
+      </c>
+      <c r="J39" t="s">
+        <v>21</v>
+      </c>
+      <c r="L39">
         <v>16.55</v>
       </c>
-      <c r="K39">
+      <c r="M39">
         <v>16.05</v>
       </c>
-      <c r="L39">
+      <c r="N39">
         <v>17.9</v>
       </c>
-      <c r="M39">
+      <c r="O39">
         <v>18.95</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B40" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C40" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D40" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E40">
         <v>16.1</v>
       </c>
       <c r="F40">
+        <v>13.1</v>
+      </c>
+      <c r="G40">
+        <v>20.15</v>
+      </c>
+      <c r="H40">
         <v>9300</v>
       </c>
-      <c r="G40" t="s">
-        <v>24</v>
-      </c>
-      <c r="H40" t="s">
-        <v>19</v>
-      </c>
-      <c r="J40">
+      <c r="I40" t="s">
+        <v>26</v>
+      </c>
+      <c r="J40" t="s">
+        <v>21</v>
+      </c>
+      <c r="L40">
         <v>16.55</v>
       </c>
-      <c r="K40">
+      <c r="M40">
         <v>16.05</v>
       </c>
-      <c r="L40">
+      <c r="N40">
         <v>17.9</v>
       </c>
-      <c r="M40">
+      <c r="O40">
         <v>18.95</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B41" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C41" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D41" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E41">
         <v>17.2</v>
       </c>
       <c r="F41">
+        <v>13.1</v>
+      </c>
+      <c r="G41">
+        <v>20.15</v>
+      </c>
+      <c r="H41">
         <v>9620</v>
       </c>
-      <c r="G41" t="s">
-        <v>18</v>
-      </c>
-      <c r="H41" t="s">
-        <v>19</v>
-      </c>
-      <c r="J41">
+      <c r="I41" t="s">
+        <v>20</v>
+      </c>
+      <c r="J41" t="s">
+        <v>21</v>
+      </c>
+      <c r="L41">
         <v>16.55</v>
       </c>
-      <c r="K41">
+      <c r="M41">
         <v>16.05</v>
       </c>
-      <c r="L41">
+      <c r="N41">
         <v>17.9</v>
       </c>
-      <c r="M41">
+      <c r="O41">
         <v>18.95</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B42" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C42" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D42" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E42">
         <v>15.2</v>
       </c>
       <c r="F42">
+        <v>13.1</v>
+      </c>
+      <c r="G42">
+        <v>20.15</v>
+      </c>
+      <c r="H42">
         <v>9950</v>
       </c>
-      <c r="G42" t="s">
-        <v>24</v>
-      </c>
-      <c r="H42" t="s">
-        <v>19</v>
-      </c>
-      <c r="J42">
+      <c r="I42" t="s">
+        <v>26</v>
+      </c>
+      <c r="J42" t="s">
+        <v>21</v>
+      </c>
+      <c r="L42">
         <v>16.55</v>
       </c>
-      <c r="K42">
+      <c r="M42">
         <v>16.05</v>
       </c>
-      <c r="L42">
+      <c r="N42">
         <v>17.9</v>
       </c>
-      <c r="M42">
+      <c r="O42">
         <v>18.95</v>
       </c>
     </row>
     <row r="43">
       <c r="F43">
+        <v>12.4</v>
+      </c>
+      <c r="G43">
+        <v>19.4</v>
+      </c>
+      <c r="H43">
         <v>10050</v>
       </c>
-      <c r="I43" t="s">
-        <v>140</v>
-      </c>
-      <c r="J43">
+      <c r="K43" t="s">
+        <v>142</v>
+      </c>
+      <c r="L43">
         <v>15.8</v>
       </c>
-      <c r="K43">
+      <c r="M43">
         <v>15.3</v>
       </c>
-      <c r="L43">
+      <c r="N43">
         <v>17.1</v>
       </c>
-      <c r="M43">
+      <c r="O43">
         <v>18.25</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B44" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C44" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D44" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E44">
         <v>15.75</v>
       </c>
       <c r="F44">
+        <v>12.4</v>
+      </c>
+      <c r="G44">
+        <v>19.4</v>
+      </c>
+      <c r="H44">
         <v>10280</v>
       </c>
-      <c r="G44" t="s">
-        <v>24</v>
-      </c>
-      <c r="H44" t="s">
-        <v>19</v>
-      </c>
-      <c r="J44">
+      <c r="I44" t="s">
+        <v>26</v>
+      </c>
+      <c r="J44" t="s">
+        <v>21</v>
+      </c>
+      <c r="L44">
         <v>15.8</v>
       </c>
-      <c r="K44">
+      <c r="M44">
         <v>15.3</v>
       </c>
-      <c r="L44">
+      <c r="N44">
         <v>17.1</v>
       </c>
-      <c r="M44">
+      <c r="O44">
         <v>18.25</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B45" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C45" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D45" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E45">
         <v>17.05</v>
       </c>
       <c r="F45">
+        <v>12.4</v>
+      </c>
+      <c r="G45">
+        <v>19.4</v>
+      </c>
+      <c r="H45">
         <v>10610</v>
       </c>
-      <c r="G45" t="s">
-        <v>24</v>
-      </c>
-      <c r="H45" t="s">
-        <v>19</v>
-      </c>
-      <c r="J45">
+      <c r="I45" t="s">
+        <v>26</v>
+      </c>
+      <c r="J45" t="s">
+        <v>21</v>
+      </c>
+      <c r="L45">
         <v>15.8</v>
       </c>
-      <c r="K45">
+      <c r="M45">
         <v>15.3</v>
       </c>
-      <c r="L45">
+      <c r="N45">
         <v>17.1</v>
       </c>
-      <c r="M45">
+      <c r="O45">
         <v>18.25</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B46" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C46" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D46" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E46">
         <v>14.1</v>
       </c>
       <c r="F46">
+        <v>12.4</v>
+      </c>
+      <c r="G46">
+        <v>19.4</v>
+      </c>
+      <c r="H46">
         <v>10940</v>
       </c>
-      <c r="G46" t="s">
-        <v>18</v>
-      </c>
-      <c r="H46" t="s">
-        <v>19</v>
-      </c>
-      <c r="J46">
+      <c r="I46" t="s">
+        <v>20</v>
+      </c>
+      <c r="J46" t="s">
+        <v>21</v>
+      </c>
+      <c r="L46">
         <v>15.8</v>
       </c>
-      <c r="K46">
+      <c r="M46">
         <v>15.3</v>
       </c>
-      <c r="L46">
+      <c r="N46">
         <v>17.1</v>
       </c>
-      <c r="M46">
+      <c r="O46">
         <v>18.25</v>
       </c>
     </row>
     <row r="47">
       <c r="F47">
+        <v>11.85</v>
+      </c>
+      <c r="G47">
+        <v>18.5</v>
+      </c>
+      <c r="H47">
         <v>11250</v>
       </c>
-      <c r="I47" t="s">
-        <v>150</v>
-      </c>
-      <c r="J47">
+      <c r="K47" t="s">
+        <v>152</v>
+      </c>
+      <c r="L47">
         <v>15.1</v>
       </c>
-      <c r="K47">
+      <c r="M47">
         <v>14.65</v>
       </c>
-      <c r="L47">
+      <c r="N47">
         <v>16.1</v>
       </c>
-      <c r="M47">
+      <c r="O47">
         <v>17.2</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B48" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C48" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D48" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E48">
         <v>14.9</v>
       </c>
       <c r="F48">
+        <v>11.85</v>
+      </c>
+      <c r="G48">
+        <v>18.5</v>
+      </c>
+      <c r="H48">
         <v>11270</v>
       </c>
-      <c r="G48" t="s">
-        <v>24</v>
-      </c>
-      <c r="H48" t="s">
-        <v>19</v>
-      </c>
-      <c r="J48">
+      <c r="I48" t="s">
+        <v>26</v>
+      </c>
+      <c r="J48" t="s">
+        <v>21</v>
+      </c>
+      <c r="L48">
         <v>15.1</v>
       </c>
-      <c r="K48">
+      <c r="M48">
         <v>14.65</v>
       </c>
-      <c r="L48">
+      <c r="N48">
         <v>16.1</v>
       </c>
-      <c r="M48">
+      <c r="O48">
         <v>17.2</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B49" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C49" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D49" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E49">
         <v>15.4</v>
       </c>
       <c r="F49">
+        <v>11.85</v>
+      </c>
+      <c r="G49">
+        <v>18.5</v>
+      </c>
+      <c r="H49">
         <v>11600</v>
       </c>
-      <c r="G49" t="s">
-        <v>18</v>
-      </c>
-      <c r="H49" t="s">
-        <v>19</v>
-      </c>
-      <c r="J49">
+      <c r="I49" t="s">
+        <v>20</v>
+      </c>
+      <c r="J49" t="s">
+        <v>21</v>
+      </c>
+      <c r="L49">
         <v>15.1</v>
       </c>
-      <c r="K49">
+      <c r="M49">
         <v>14.65</v>
       </c>
-      <c r="L49">
+      <c r="N49">
         <v>16.1</v>
       </c>
-      <c r="M49">
+      <c r="O49">
         <v>17.2</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B50" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C50" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D50" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E50">
         <v>14.1</v>
       </c>
       <c r="F50">
+        <v>11.85</v>
+      </c>
+      <c r="G50">
+        <v>18.5</v>
+      </c>
+      <c r="H50">
         <v>11880</v>
       </c>
-      <c r="G50" t="s">
-        <v>18</v>
-      </c>
-      <c r="H50" t="s">
-        <v>19</v>
-      </c>
-      <c r="J50">
+      <c r="I50" t="s">
+        <v>20</v>
+      </c>
+      <c r="J50" t="s">
+        <v>21</v>
+      </c>
+      <c r="L50">
         <v>15.1</v>
       </c>
-      <c r="K50">
+      <c r="M50">
         <v>14.65</v>
       </c>
-      <c r="L50">
+      <c r="N50">
         <v>16.1</v>
       </c>
-      <c r="M50">
+      <c r="O50">
         <v>17.2</v>
       </c>
     </row>
     <row r="51">
       <c r="F51">
+        <v>11.6</v>
+      </c>
+      <c r="G51">
+        <v>18.15</v>
+      </c>
+      <c r="H51">
         <v>12000</v>
       </c>
-      <c r="I51" t="s">
-        <v>160</v>
-      </c>
-      <c r="J51">
+      <c r="K51" t="s">
+        <v>162</v>
+      </c>
+      <c r="L51">
         <v>14.9</v>
       </c>
-      <c r="K51">
+      <c r="M51">
         <v>14.4</v>
       </c>
-      <c r="L51">
+      <c r="N51">
         <v>15.8</v>
       </c>
-      <c r="M51">
+      <c r="O51">
         <v>16.9</v>
       </c>
     </row>

</xml_diff>